<commit_message>
modf rout et affair.js
</commit_message>
<xml_diff>
--- a/scripts/files/2024_t2_sites_metropoles_bis.xlsx
+++ b/scripts/files/2024_t2_sites_metropoles_bis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fomnenkam\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CrimeLab\scripts\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B8CB109-F9B6-42BC-9FA4-FF5A83F0998E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79534D1C-8DC8-4939-82DC-36FF5248B28C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{97D5244B-6D0A-4F3A-A10B-052B99C93C2A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{97D5244B-6D0A-4F3A-A10B-052B99C93C2A}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -1051,9 +1051,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE5BADC7-609C-46E0-9A67-5A374BCF81EB}">
   <dimension ref="A1:AC52"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="11" max="11" width="26.6328125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1142,7 +1145,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>20801</v>
       </c>
@@ -1225,7 +1228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>20801</v>
       </c>
@@ -1311,7 +1314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>20801</v>
       </c>
@@ -1397,7 +1400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>20801</v>
       </c>
@@ -1483,7 +1486,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>20801</v>
       </c>
@@ -1566,7 +1569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>20801</v>
       </c>
@@ -1649,7 +1652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>20801</v>
       </c>
@@ -1735,7 +1738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>20801</v>
       </c>
@@ -1821,7 +1824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>20801</v>
       </c>
@@ -1907,7 +1910,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>20801</v>
       </c>
@@ -1993,7 +1996,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>20810</v>
       </c>
@@ -2076,7 +2079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>20810</v>
       </c>
@@ -2162,7 +2165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>20810</v>
       </c>
@@ -2248,7 +2251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>20810</v>
       </c>
@@ -2334,7 +2337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>20810</v>
       </c>
@@ -2420,7 +2423,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>20810</v>
       </c>
@@ -2506,7 +2509,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>20810</v>
       </c>
@@ -2592,7 +2595,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>20810</v>
       </c>
@@ -2678,7 +2681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>20810</v>
       </c>
@@ -2764,7 +2767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20810</v>
       </c>
@@ -2850,7 +2853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>20810</v>
       </c>
@@ -2936,7 +2939,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>20810</v>
       </c>
@@ -3019,7 +3022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>20810</v>
       </c>
@@ -3105,7 +3108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>20810</v>
       </c>
@@ -3188,7 +3191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>20810</v>
       </c>
@@ -3274,7 +3277,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>20810</v>
       </c>
@@ -3357,7 +3360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>20820</v>
       </c>
@@ -3443,7 +3446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>20820</v>
       </c>
@@ -3529,7 +3532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>20820</v>
       </c>
@@ -3615,7 +3618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>20820</v>
       </c>
@@ -3701,7 +3704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>20820</v>
       </c>
@@ -3787,7 +3790,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>20820</v>
       </c>
@@ -3873,7 +3876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>20820</v>
       </c>
@@ -3959,7 +3962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>20820</v>
       </c>
@@ -4045,7 +4048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>20820</v>
       </c>
@@ -4131,7 +4134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>20820</v>
       </c>
@@ -4217,7 +4220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>20820</v>
       </c>
@@ -4303,7 +4306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>20815</v>
       </c>
@@ -4389,7 +4392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>20815</v>
       </c>
@@ -4475,7 +4478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>20815</v>
       </c>
@@ -4561,7 +4564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>20815</v>
       </c>
@@ -4647,7 +4650,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>20815</v>
       </c>
@@ -4733,7 +4736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>20815</v>
       </c>
@@ -4819,7 +4822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>20815</v>
       </c>
@@ -4905,7 +4908,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>20815</v>
       </c>
@@ -4991,7 +4994,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>20815</v>
       </c>
@@ -5077,7 +5080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>20815</v>
       </c>
@@ -5163,7 +5166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>20815</v>
       </c>
@@ -5249,7 +5252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>20801</v>
       </c>
@@ -5332,7 +5335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>20815</v>
       </c>
@@ -5415,7 +5418,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>20810</v>
       </c>

</xml_diff>